<commit_message>
dev-opencode: added analysis column
</commit_message>
<xml_diff>
--- a/tests/fixtures/reference/Test_Range_Merged.xlsx
+++ b/tests/fixtures/reference/Test_Range_Merged.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -11,7 +11,7 @@
     <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">#REF!</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">#ref!</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -228,37 +228,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Оffice">
@@ -397,284 +397,302 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:XFD29"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.84"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="7" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16365" min="14" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16366" style="1" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7.84"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="8" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16366" min="15" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16367" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E2" s="4"/>
+      <c r="D2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="G3" s="1"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
     </row>
     <row r="4" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E4" s="4"/>
+      <c r="D4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F4" s="4"/>
-      <c r="G4" s="1"/>
+      <c r="G4" s="4"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="2"/>
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E5" s="4"/>
+      <c r="D5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E6" s="4"/>
+      <c r="D6" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2"/>
+      <c r="C7" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="2"/>
+      <c r="C8" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E8" s="4"/>
+      <c r="D8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2"/>
+      <c r="C9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
-      <c r="G9" s="1"/>
+      <c r="G9" s="4"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
     </row>
     <row r="10" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="2"/>
+      <c r="C10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E10" s="4"/>
+      <c r="D10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F10" s="4"/>
-      <c r="G10" s="1"/>
+      <c r="G10" s="4"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="2"/>
+      <c r="C11" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E11" s="4"/>
+      <c r="D11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="2"/>
+      <c r="C12" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E12" s="4"/>
+      <c r="D12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2"/>
+      <c r="C13" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="2"/>
+      <c r="C14" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E14" s="4"/>
+      <c r="D14" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="2"/>
+      <c r="C15" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" s="4" t="n">
         <v>999</v>
       </c>
-      <c r="E15" s="4"/>
       <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
     </row>
     <row r="16" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2"/>
+      <c r="C16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-      <c r="G16" s="1"/>
+      <c r="G16" s="4"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
     </row>
     <row r="17" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="2"/>
+      <c r="C17" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E17" s="4"/>
+      <c r="D17" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F17" s="4"/>
-      <c r="G17" s="1"/>
+      <c r="G17" s="4"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="2"/>
+      <c r="C18" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E18" s="4"/>
+      <c r="D18" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F18" s="4"/>
-      <c r="XEL18" s="6"/>
+      <c r="G18" s="4"/>
       <c r="XEM18" s="6"/>
       <c r="XEN18" s="6"/>
       <c r="XEO18" s="6"/>
@@ -698,213 +716,169 @@
       <c r="A19" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="2"/>
+      <c r="C19" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
-      <c r="G19" s="1"/>
+      <c r="G19" s="4"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
     </row>
     <row r="20" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="2"/>
+      <c r="C20" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="4"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="1"/>
+      <c r="G20" s="4"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="2"/>
+      <c r="C21" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="4"/>
+      <c r="D21" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2"/>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="2"/>
+      <c r="C22" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D22" s="4" t="n">
+      <c r="D22" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="4"/>
       <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="2"/>
+      <c r="C23" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="2"/>
+      <c r="C24" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E24" s="4"/>
+      <c r="D24" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="2"/>
+      <c r="C25" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" s="4" t="n">
+      <c r="D25" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E25" s="4" t="n">
         <v>888</v>
       </c>
-      <c r="E25" s="4"/>
       <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="2"/>
+      <c r="C26" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D26" s="4" t="n">
+      <c r="D26" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="4" t="n">
         <v>777</v>
       </c>
-      <c r="E26" s="4"/>
       <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2"/>
+      <c r="C27" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="4"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="2"/>
+      <c r="C28" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E28" s="4"/>
+      <c r="D28" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2"/>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="2"/>
+      <c r="C29" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D29" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E29" s="4"/>
+      <c r="D29" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="F29" s="4"/>
-    </row>
-    <row r="1048522" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048523" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048524" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048525" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048526" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048527" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048528" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048529" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048530" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048531" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048532" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048533" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048534" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048535" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048536" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048537" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048538" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048539" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048540" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048541" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048542" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048543" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048544" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048545" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048546" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048547" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048548" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048549" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048550" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048551" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048552" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048553" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="G29" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:A2"/>

</xml_diff>